<commit_message>
Fixed the code for date which caused issues, create a new file to ensure WriteDB and SendEmail work from any script
</commit_message>
<xml_diff>
--- a/interview_database.xlsx
+++ b/interview_database.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +28,14 @@
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -62,19 +70,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -442,8 +453,8 @@
   <cols>
     <col width="13.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="37.140625" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="17.85546875" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="8.5703125" customWidth="1" min="7" max="7"/>
+    <col width="31" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="73.42578125" bestFit="1" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -558,12 +569,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Zoz, Alice Johnson, Charlie Brown</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Zoz@example.com, darkicewolf50@gmail.com, charlie.brown@example.com</t>
+          <t>Alice Johnson</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>ahmadmuhammadofficial@gmail.com</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -741,16 +752,6 @@
       </c>
       <c r="C9" s="3" t="n">
         <v>0.5625</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Bob Smith</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>ahmadmuhammadofficial@gmail.com</t>
-        </is>
       </c>
       <c r="I9" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
feat(putTogether): read db also combined
</commit_message>
<xml_diff>
--- a/interview_database.xlsx
+++ b/interview_database.xlsx
@@ -568,12 +568,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Zoz, Alice Johnson, Alice Johnson</t>
+          <t>Zoz, Alice Johnson, Alice Johnson, Alice Johnson, Alice Johnson, Alice Johnson, Alice Johnson, Alice Johnson</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Zoz@example.com, ahmadmuhammadofficial@gmail.com, darkicewolf50@gmail.com</t>
+          <t>Zoz@example.com, ahmadmuhammadofficial@gmail.com, darkicewolf50@gmail.com, darkicewolf50@gmail.com, darkicewolf50@gmail.coaaaa, darkicewolf50@gma.com, darkicewolf50@gma.com, darkicewolf50@gma.com</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">

</xml_diff>